<commit_message>
Add leaderboard feature with dynamic data fetching and display
</commit_message>
<xml_diff>
--- a/JAMB Slips (version 2).xlsx
+++ b/JAMB Slips (version 2).xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\JAMB_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6BF8D41-27CC-430C-AE63-5A2A1BDB2BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3A2781E-1791-48C5-87F9-F35BD5D6A288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{6CD54D3B-EF31-4377-8F6B-04DD1C271DA9}"/>
+    <workbookView xWindow="33450" yWindow="1770" windowWidth="17280" windowHeight="9420" xr2:uid="{6CD54D3B-EF31-4377-8F6B-04DD1C271DA9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2564,10 +2563,10 @@
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A194" t="s">
+      <c r="A194" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B194">
+      <c r="B194" s="1">
         <v>6059</v>
       </c>
     </row>

</xml_diff>